<commit_message>
Final review pass: coherence, fact-check corrections and budget alignment
</commit_message>
<xml_diff>
--- a/docs/phase-1/Relivable Feature Matrix.xlsx
+++ b/docs/phase-1/Relivable Feature Matrix.xlsx
@@ -423,7 +423,7 @@
     <t xml:space="preserve">Seed codes (generate, enter, share, QR)</t>
   </si>
   <si>
-    <t xml:space="preserve">Human-readable EL- seed on Review, death screen and recap; reproduces the start</t>
+    <t xml:space="preserve">Human-readable #RL- seed on Review, death screen and recap; reproduces the start</t>
   </si>
   <si>
     <t xml:space="preserve">CORE-CL, SOC-CE</t>
@@ -5019,7 +5019,7 @@
     <t xml:space="preserve">Short server share codes and deep links</t>
   </si>
   <si>
-    <t xml:space="preserve">EL- codes mapped to a server record; deep links and web links</t>
+    <t xml:space="preserve">#RL- codes mapped to a server record; deep links and web links</t>
   </si>
   <si>
     <t xml:space="preserve">No share code system</t>
@@ -6381,19 +6381,19 @@
     <t xml:space="preserve">Phase 5 LiveOps run rate (per month)</t>
   </si>
   <si>
-    <t xml:space="preserve">Low (LatAm, 6 FTE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High (EE, 8 FTE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US ref (7 FTE)</t>
+    <t xml:space="preserve">Low (LatAm, 7.5 FTE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High (EE, 9.0 FTE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US ref (8.25 FTE)</t>
   </si>
   <si>
     <t xml:space="preserve">Phase 5 LiveOps (monthly)</t>
   </si>
   <si>
-    <t xml:space="preserve">Labour (960-1,280 h)</t>
+    <t xml:space="preserve">Labour (1,200-1,440 h)</t>
   </si>
   <si>
     <t xml:space="preserve">Services (Firebase, Crowdin, MMP, CI, ASO tool)</t>
@@ -6507,7 +6507,7 @@
     <t xml:space="preserve">5 LiveOps</t>
   </si>
   <si>
-    <t xml:space="preserve">6-8</t>
+    <t xml:space="preserve">7.5-9.0</t>
   </si>
   <si>
     <t xml:space="preserve">Gate 5: launch + 90 days (Jan 2028); quarterly reviews</t>
@@ -6609,7 +6609,7 @@
     <t xml:space="preserve">Weekly challenges + seasons</t>
   </si>
   <si>
-    <t xml:space="preserve">Story Packs (quarterly)</t>
+    <t xml:space="preserve">Story Packs (every 2 months)</t>
   </si>
   <si>
     <t xml:space="preserve">Async social</t>
@@ -30432,13 +30432,13 @@
         <v>2120</v>
       </c>
       <c r="C32" s="27" t="n">
-        <v>48000</v>
+        <v>60000</v>
       </c>
       <c r="D32" s="27" t="n">
-        <v>77000</v>
+        <v>86000</v>
       </c>
       <c r="E32" s="27" t="n">
-        <v>123000</v>
+        <v>145000</v>
       </c>
       <c r="F32" s="33"/>
       <c r="G32" s="33"/>
@@ -30490,15 +30490,15 @@
       </c>
       <c r="C35" s="29" t="n">
         <f aca="false">SUM(C32:C34)</f>
-        <v>54000</v>
+        <v>66000</v>
       </c>
       <c r="D35" s="29" t="n">
         <f aca="false">SUM(D32:D34)</f>
-        <v>90000</v>
+        <v>99000</v>
       </c>
       <c r="E35" s="29" t="n">
         <f aca="false">SUM(E32:E34)</f>
-        <v>136000</v>
+        <v>158000</v>
       </c>
       <c r="F35" s="28"/>
       <c r="G35" s="28"/>
@@ -30512,15 +30512,15 @@
       </c>
       <c r="C36" s="34" t="n">
         <f aca="false">C35*12</f>
-        <v>648000</v>
+        <v>792000</v>
       </c>
       <c r="D36" s="34" t="n">
         <f aca="false">D35*12</f>
-        <v>1080000</v>
+        <v>1188000</v>
       </c>
       <c r="E36" s="34" t="n">
         <f aca="false">E35*12</f>
-        <v>1632000</v>
+        <v>1896000</v>
       </c>
       <c r="F36" s="21"/>
       <c r="G36" s="21"/>
@@ -31289,7 +31289,7 @@
         <v>2166</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
         <v>2157</v>
       </c>

</xml_diff>

<commit_message>
Make world history one world per player with one continuous history
</commit_message>
<xml_diff>
--- a/docs/phase-1/Relivable Feature Matrix.xlsx
+++ b/docs/phase-1/Relivable Feature Matrix.xlsx
@@ -3330,7 +3330,7 @@
     <t xml:space="preserve">World Ledger</t>
   </si>
   <si>
-    <t xml:space="preserve">Persistent record of notable people, companies, landmarks, laws and events, shared by all dynasties in a world (cap about 250 entries)</t>
+    <t xml:space="preserve">Persistent record of notable people, companies, landmarks, laws and events, shared by every life and dynasty in the player's one world (cap about 250 active entries)</t>
   </si>
   <si>
     <t xml:space="preserve">CORE-WL-008</t>
@@ -3423,10 +3423,10 @@
     <t xml:space="preserve">CORE-WL-016</t>
   </si>
   <si>
-    <t xml:space="preserve">New world option</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Start a fresh world at any time so no history traps the player</t>
+    <t xml:space="preserve">One world, one continuous history</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every life and dynasty a player ever plays shares one persistent world and Ledger that is never reset; a life only sees history dated before its current year</t>
   </si>
   <si>
     <t xml:space="preserve">CORE-WL-017</t>
@@ -19229,7 +19229,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="253" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="253" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="10" t="s">
         <v>1129</v>
       </c>
@@ -19249,13 +19249,13 @@
         <v>105</v>
       </c>
       <c r="G253" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H253" s="11" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="I253" s="11" t="s">
-        <v>144</v>
+        <v>106</v>
       </c>
       <c r="J253" s="11" t="s">
         <v>91</v>
@@ -29140,11 +29140,11 @@
       </c>
       <c r="C16" s="15" t="n">
         <f aca="false">COUNTIFS('Feature Matrix'!$B$2:$B$1000,$A16,'Feature Matrix'!$I$2:$I$1000,C$5)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D16" s="15" t="n">
         <f aca="false">COUNTIFS('Feature Matrix'!$B$2:$B$1000,$A16,'Feature Matrix'!$I$2:$I$1000,D$5)</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E16" s="15" t="n">
         <f aca="false">COUNTIFS('Feature Matrix'!$B$2:$B$1000,$A16,'Feature Matrix'!$I$2:$I$1000,E$5)</f>
@@ -29156,7 +29156,7 @@
       </c>
       <c r="G16" s="16" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Feature Matrix'!$G$2:$G$1000,'Feature Matrix'!$B$2:$B$1000,$A16),0)</f>
-        <v>3.84210526315789</v>
+        <v>3.94736842105263</v>
       </c>
       <c r="H16" s="15" t="n">
         <f aca="false">COUNTIFS('Feature Matrix'!$B$2:$B$1000,$A16,'Feature Matrix'!$J$2:$J$1000,"Free")</f>
@@ -29755,11 +29755,11 @@
       </c>
       <c r="C31" s="17" t="n">
         <f aca="false">SUM(C6:C30)</f>
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D31" s="17" t="n">
         <f aca="false">SUM(D6:D30)</f>
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E31" s="17" t="n">
         <f aca="false">SUM(E6:E30)</f>
@@ -29771,7 +29771,7 @@
       </c>
       <c r="G31" s="18" t="n">
         <f aca="false">IFERROR(AVERAGE('Feature Matrix'!$G$2:$G$1000),0)</f>
-        <v>3.35490605427975</v>
+        <v>3.35908141962422</v>
       </c>
       <c r="H31" s="17" t="n">
         <f aca="false">SUM(H6:H30)</f>
@@ -29905,11 +29905,11 @@
       </c>
       <c r="C43" s="14" t="n">
         <f aca="false">COUNTIFS('Feature Matrix'!$J$2:$J$1000,$A43,'Feature Matrix'!$I$2:$I$1000,C$42)</f>
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D43" s="14" t="n">
         <f aca="false">COUNTIFS('Feature Matrix'!$J$2:$J$1000,$A43,'Feature Matrix'!$I$2:$I$1000,D$42)</f>
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E43" s="14" t="n">
         <f aca="false">COUNTIFS('Feature Matrix'!$J$2:$J$1000,$A43,'Feature Matrix'!$I$2:$I$1000,E$42)</f>
@@ -30050,11 +30050,11 @@
       </c>
       <c r="C48" s="21" t="n">
         <f aca="false">SUM(C43:C47)</f>
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D48" s="21" t="n">
         <f aca="false">SUM(D43:D47)</f>
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E48" s="21" t="n">
         <f aca="false">SUM(E43:E47)</f>

</xml_diff>